<commit_message>
Modelos de prediccion terminados
</commit_message>
<xml_diff>
--- a/data/inputs/trabajadores.xlsx
+++ b/data/inputs/trabajadores.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/jaimeteran/Documents/PYTHON/VacanzeGIT/data/inputs/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{718B0742-88D6-7547-A06A-A3826AB3158E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{80033505-91EE-2C4C-918E-C107D2F195F1}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="18000" yWindow="660" windowWidth="11400" windowHeight="17140" xr2:uid="{93ADCB3C-DA1B-7146-A2FE-0804F0036F5D}"/>
   </bookViews>
@@ -1235,7 +1235,7 @@
         <v>36</v>
       </c>
       <c r="E31">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="F31">
         <v>1</v>
@@ -1252,7 +1252,7 @@
         <v>37</v>
       </c>
       <c r="E32">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="F32">
         <v>1</v>
@@ -1269,7 +1269,7 @@
         <v>38</v>
       </c>
       <c r="E33">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="F33">
         <v>1</v>
@@ -1286,7 +1286,7 @@
         <v>39</v>
       </c>
       <c r="E34">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="F34">
         <v>0</v>
@@ -1303,7 +1303,7 @@
         <v>40</v>
       </c>
       <c r="E35">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="F35">
         <v>0</v>
@@ -1320,7 +1320,7 @@
         <v>41</v>
       </c>
       <c r="E36">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="F36">
         <v>0</v>
@@ -1337,7 +1337,7 @@
         <v>42</v>
       </c>
       <c r="E37">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="F37">
         <v>1</v>
@@ -1354,7 +1354,7 @@
         <v>43</v>
       </c>
       <c r="E38">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="F38">
         <v>1</v>
@@ -1371,7 +1371,7 @@
         <v>44</v>
       </c>
       <c r="E39">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="F39">
         <v>1</v>
@@ -1388,7 +1388,7 @@
         <v>45</v>
       </c>
       <c r="E40">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="F40">
         <v>1</v>
@@ -1405,7 +1405,7 @@
         <v>40</v>
       </c>
       <c r="E41">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="F41">
         <v>1</v>
@@ -1422,7 +1422,7 @@
         <v>41</v>
       </c>
       <c r="E42">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="F42">
         <v>1</v>

</xml_diff>

<commit_message>
xgboost y correccion de predictor
</commit_message>
<xml_diff>
--- a/data/inputs/trabajadores.xlsx
+++ b/data/inputs/trabajadores.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/jaimeteran/Documents/PYTHON/VacanzeGIT/data/inputs/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{7087BC31-9EFF-A946-BC76-85EB02171240}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{CE707020-2150-B74C-A47C-3C3B785A061D}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="18000" yWindow="660" windowWidth="11400" windowHeight="17140" xr2:uid="{93ADCB3C-DA1B-7146-A2FE-0804F0036F5D}"/>
   </bookViews>
@@ -1235,7 +1235,7 @@
         <v>36</v>
       </c>
       <c r="E31">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="F31">
         <v>1</v>
@@ -1252,7 +1252,7 @@
         <v>37</v>
       </c>
       <c r="E32">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="F32">
         <v>1</v>
@@ -1269,7 +1269,7 @@
         <v>38</v>
       </c>
       <c r="E33">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="F33">
         <v>1</v>
@@ -1286,7 +1286,7 @@
         <v>39</v>
       </c>
       <c r="E34">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="F34">
         <v>0</v>
@@ -1303,7 +1303,7 @@
         <v>40</v>
       </c>
       <c r="E35">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="F35">
         <v>0</v>
@@ -1320,7 +1320,7 @@
         <v>41</v>
       </c>
       <c r="E36">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="F36">
         <v>0</v>
@@ -1337,7 +1337,7 @@
         <v>42</v>
       </c>
       <c r="E37">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="F37">
         <v>1</v>
@@ -1354,7 +1354,7 @@
         <v>43</v>
       </c>
       <c r="E38">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="F38">
         <v>1</v>
@@ -1371,7 +1371,7 @@
         <v>44</v>
       </c>
       <c r="E39">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="F39">
         <v>1</v>
@@ -1388,7 +1388,7 @@
         <v>45</v>
       </c>
       <c r="E40">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="F40">
         <v>1</v>
@@ -1405,7 +1405,7 @@
         <v>40</v>
       </c>
       <c r="E41">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="F41">
         <v>1</v>
@@ -1422,7 +1422,7 @@
         <v>41</v>
       </c>
       <c r="E42">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="F42">
         <v>1</v>

</xml_diff>